<commit_message>
Migrate domain to brand-first reputetap.github.io, update all demo links and WhatsApp prefilled outreach messages
</commit_message>
<xml_diff>
--- a/ReputeTap - 100 Outreach Leads (Vadodara & Gujarat).xlsx
+++ b/ReputeTap - 100 Outreach Leads (Vadodara & Gujarat).xlsx
@@ -457,12 +457,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=curators-coffee</t>
+          <t>https://reputetap.github.io/?id=curators-coffee</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/916359220791?text=Hi%20Curators%20Coffee%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Curators%20Coffee%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcurators-coffee%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/916359220791?text=Hi%20Curators%20Coffee%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Curators%20Coffee%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcurators-coffee%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -502,12 +502,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=kaffa-coffee-roasters</t>
+          <t>https://reputetap.github.io/?id=kaffa-coffee-roasters</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825336364?text=Hi%20Kaffa%20Coffee%20Roasters%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kaffa%20Coffee%20Roasters%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dkaffa-coffee-roasters%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825336364?text=Hi%20Kaffa%20Coffee%20Roasters%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kaffa%20Coffee%20Roasters%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkaffa-coffee-roasters%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -547,12 +547,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-coffee-next-door</t>
+          <t>https://reputetap.github.io/?id=the-coffee-next-door</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919978623256?text=Hi%20The%20Coffee%20Next%20Door%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Coffee%20Next%20Door%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-coffee-next-door%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919978623256?text=Hi%20The%20Coffee%20Next%20Door%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Coffee%20Next%20Door%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-coffee-next-door%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -592,12 +592,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=charmant-the-heritage-caf</t>
+          <t>https://reputetap.github.io/?id=charmant-the-heritage-caf</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919773050954?text=Hi%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcharmant-the-heritage-caf%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919773050954?text=Hi%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcharmant-the-heritage-caf%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -637,12 +637,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=burgundy-cafe</t>
+          <t>https://reputetap.github.io/?id=burgundy-cafe</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/916357575811?text=Hi%20Burgundy%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Burgundy%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dburgundy-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/916357575811?text=Hi%20Burgundy%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Burgundy%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dburgundy-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -682,12 +682,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=trinity-cafe</t>
+          <t>https://reputetap.github.io/?id=trinity-cafe</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919712348900?text=Hi%20Trinity%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Trinity%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dtrinity-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919712348900?text=Hi%20Trinity%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Trinity%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtrinity-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -727,12 +727,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-dark-roast</t>
+          <t>https://reputetap.github.io/?id=the-dark-roast</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123451?text=Hi%20The%20Dark%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dark%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-dark-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123451?text=Hi%20The%20Dark%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dark%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dark-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=brew-artisan-cafe</t>
+          <t>https://reputetap.github.io/?id=brew-artisan-cafe</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123452?text=Hi%20Brew%20Artisan%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Brew%20Artisan%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dbrew-artisan-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123452?text=Hi%20Brew%20Artisan%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Brew%20Artisan%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbrew-artisan-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=mocha-vadodara</t>
+          <t>https://reputetap.github.io/?id=mocha-vadodara</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123453?text=Hi%20Mocha%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mocha%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dmocha-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123453?text=Hi%20Mocha%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mocha%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmocha-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=cafe-fitoor</t>
+          <t>https://reputetap.github.io/?id=cafe-fitoor</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123454?text=Hi%20Cafe%20Fitoor%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cafe%20Fitoor%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcafe-fitoor%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123454?text=Hi%20Cafe%20Fitoor%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cafe%20Fitoor%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcafe-fitoor%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-secret-kitchen</t>
+          <t>https://reputetap.github.io/?id=the-secret-kitchen</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123455?text=Hi%20The%20Secret%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Secret%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-secret-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123455?text=Hi%20The%20Secret%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Secret%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-secret-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=kai-asia</t>
+          <t>https://reputetap.github.io/?id=kai-asia</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123456?text=Hi%20Kai%20Asia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kai%20Asia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dkai-asia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123456?text=Hi%20Kai%20Asia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kai%20Asia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkai-asia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=gazebo-garden-restaurant</t>
+          <t>https://reputetap.github.io/?id=gazebo-garden-restaurant</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123457?text=Hi%20Gazebo%20Garden%20Restaurant%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gazebo%20Garden%20Restaurant%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dgazebo-garden-restaurant%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123457?text=Hi%20Gazebo%20Garden%20Restaurant%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gazebo%20Garden%20Restaurant%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgazebo-garden-restaurant%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1042,12 +1042,12 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=little-italy</t>
+          <t>https://reputetap.github.io/?id=little-italy</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123458?text=Hi%20Little%20Italy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Little%20Italy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dlittle-italy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123458?text=Hi%20Little%20Italy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Little%20Italy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlittle-italy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1087,12 +1087,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=22nd-parallel</t>
+          <t>https://reputetap.github.io/?id=22nd-parallel</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123459?text=Hi%2022nd%20Parallel%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2022nd%20Parallel%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3D22nd-parallel%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123459?text=Hi%2022nd%20Parallel%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2022nd%20Parallel%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D22nd-parallel%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1132,12 +1132,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=salsa-kitchen</t>
+          <t>https://reputetap.github.io/?id=salsa-kitchen</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123460?text=Hi%20Salsa%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Salsa%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dsalsa-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123460?text=Hi%20Salsa%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Salsa%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsalsa-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1177,12 +1177,12 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=barbeque-nation</t>
+          <t>https://reputetap.github.io/?id=barbeque-nation</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123461?text=Hi%20Barbeque%20Nation%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Barbeque%20Nation%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dbarbeque-nation%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123461?text=Hi%20Barbeque%20Nation%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Barbeque%20Nation%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbarbeque-nation%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1222,12 +1222,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=that-place</t>
+          <t>https://reputetap.github.io/?id=that-place</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123462?text=Hi%20That%20Place%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20That%20Place%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthat-place%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123462?text=Hi%20That%20Place%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20That%20Place%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthat-place%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1267,12 +1267,12 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=fresh-roast</t>
+          <t>https://reputetap.github.io/?id=fresh-roast</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123463?text=Hi%20Fresh%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fresh%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dfresh-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123463?text=Hi%20Fresh%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fresh%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfresh-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1312,12 +1312,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=coffee-culture</t>
+          <t>https://reputetap.github.io/?id=coffee-culture</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123464?text=Hi%20Coffee%20Culture%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Coffee%20Culture%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcoffee-culture%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123464?text=Hi%20Coffee%20Culture%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Coffee%20Culture%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcoffee-culture%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=chai-sutta-bar</t>
+          <t>https://reputetap.github.io/?id=chai-sutta-bar</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123465?text=Hi%20Chai%20Sutta%20Bar%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Chai%20Sutta%20Bar%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dchai-sutta-bar%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123465?text=Hi%20Chai%20Sutta%20Bar%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Chai%20Sutta%20Bar%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchai-sutta-bar%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1402,12 +1402,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=keventers-vadodara</t>
+          <t>https://reputetap.github.io/?id=keventers-vadodara</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123466?text=Hi%20Keventers%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Keventers%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dkeventers-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123466?text=Hi%20Keventers%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Keventers%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkeventers-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1447,12 +1447,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=crust-and-crumbs-patisserie</t>
+          <t>https://reputetap.github.io/?id=crust-and-crumbs-patisserie</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123467?text=Hi%20Crust%20%26%20Crumbs%20Patisserie%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Crust%20%26%20Crumbs%20Patisserie%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcrust-and-crumbs-patisserie%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123467?text=Hi%20Crust%20%26%20Crumbs%20Patisserie%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Crust%20%26%20Crumbs%20Patisserie%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcrust-and-crumbs-patisserie%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=bake-my-day</t>
+          <t>https://reputetap.github.io/?id=bake-my-day</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123468?text=Hi%20Bake%20My%20Day%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bake%20My%20Day%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dbake-my-day%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123468?text=Hi%20Bake%20My%20Day%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bake%20My%20Day%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbake-my-day%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1537,12 +1537,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-chocolate-room</t>
+          <t>https://reputetap.github.io/?id=the-chocolate-room</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123469?text=Hi%20The%20Chocolate%20Room%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Chocolate%20Room%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-chocolate-room%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123469?text=Hi%20The%20Chocolate%20Room%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Chocolate%20Room%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-chocolate-room%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=styloria-unisex-hair-studio-and-lounge</t>
+          <t>https://reputetap.github.io/?id=styloria-unisex-hair-studio-and-lounge</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919974098750?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dstyloria-unisex-hair-studio-and-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919974098750?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio-and-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1627,12 +1627,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=styloria-unisex-hair-studio</t>
+          <t>https://reputetap.github.io/?id=styloria-unisex-hair-studio</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917600088148?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dstyloria-unisex-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/917600088148?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -1672,12 +1672,12 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=enrich-salon-vadodara</t>
+          <t>https://reputetap.github.io/?id=enrich-salon-vadodara</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919152253000?text=Hi%20Enrich%20Salon%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Enrich%20Salon%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Denrich-salon-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919152253000?text=Hi%20Enrich%20Salon%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Enrich%20Salon%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denrich-salon-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -1717,12 +1717,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=wave-salon-and-academy</t>
+          <t>https://reputetap.github.io/?id=wave-salon-and-academy</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918238307599?text=Hi%20Wave%20Salon%20%26%20Academy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Wave%20Salon%20%26%20Academy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dwave-salon-and-academy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/918238307599?text=Hi%20Wave%20Salon%20%26%20Academy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Wave%20Salon%20%26%20Academy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dwave-salon-and-academy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -1762,12 +1762,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=lakme-salon-for-him-and-her</t>
+          <t>https://reputetap.github.io/?id=lakme-salon-for-him-and-her</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918291128445?text=Hi%20Lakme%20Salon%20For%20Him%20%26%20Her%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Lakme%20Salon%20For%20Him%20%26%20Her%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dlakme-salon-for-him-and-her%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/918291128445?text=Hi%20Lakme%20Salon%20For%20Him%20%26%20Her%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Lakme%20Salon%20For%20Him%20%26%20Her%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlakme-salon-for-him-and-her%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=cutz-beauty-salon</t>
+          <t>https://reputetap.github.io/?id=cutz-beauty-salon</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/912652323222?text=Hi%20Cutz%20Beauty%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cutz%20Beauty%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcutz-beauty-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/912652323222?text=Hi%20Cutz%20Beauty%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cutz%20Beauty%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcutz-beauty-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -1852,12 +1852,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=champion-ladies-and-gents-salon</t>
+          <t>https://reputetap.github.io/?id=champion-ladies-and-gents-salon</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919724661172?text=Hi%20Champion%20Ladies%20%26%20Gents%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Champion%20Ladies%20%26%20Gents%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dchampion-ladies-and-gents-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919724661172?text=Hi%20Champion%20Ladies%20%26%20Gents%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Champion%20Ladies%20%26%20Gents%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchampion-ladies-and-gents-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -1897,12 +1897,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=truefitt-and-hill</t>
+          <t>https://reputetap.github.io/?id=truefitt-and-hill</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123470?text=Hi%20Truefitt%20%26%20Hill%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Truefitt%20%26%20Hill%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dtruefitt-and-hill%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123470?text=Hi%20Truefitt%20%26%20Hill%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Truefitt%20%26%20Hill%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtruefitt-and-hill%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=toni-and-guy</t>
+          <t>https://reputetap.github.io/?id=toni-and-guy</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123471?text=Hi%20Toni%20%26%20Guy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Toni%20%26%20Guy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dtoni-and-guy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123471?text=Hi%20Toni%20%26%20Guy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Toni%20%26%20Guy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtoni-and-guy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -1987,12 +1987,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=jawed-habib-hair-and-beauty</t>
+          <t>https://reputetap.github.io/?id=jawed-habib-hair-and-beauty</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123472?text=Hi%20Jawed%20Habib%20Hair%20%26%20Beauty%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Jawed%20Habib%20Hair%20%26%20Beauty%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Djawed-habib-hair-and-beauty%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123472?text=Hi%20Jawed%20Habib%20Hair%20%26%20Beauty%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Jawed%20Habib%20Hair%20%26%20Beauty%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djawed-habib-hair-and-beauty%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=bespoke-hair-studio</t>
+          <t>https://reputetap.github.io/?id=bespoke-hair-studio</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123473?text=Hi%20Bespoke%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bespoke%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dbespoke-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123473?text=Hi%20Bespoke%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bespoke%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbespoke-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-nail-room-baroda</t>
+          <t>https://reputetap.github.io/?id=the-nail-room-baroda</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123474?text=Hi%20The%20Nail%20Room%20Baroda%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Nail%20Room%20Baroda%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-nail-room-baroda%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123474?text=Hi%20The%20Nail%20Room%20Baroda%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Nail%20Room%20Baroda%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-nail-room-baroda%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2122,12 +2122,12 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=glam-studio</t>
+          <t>https://reputetap.github.io/?id=glam-studio</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123475?text=Hi%20Glam%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Glam%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dglam-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123475?text=Hi%20Glam%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Glam%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dglam-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2167,12 +2167,12 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=geetanjali-salon</t>
+          <t>https://reputetap.github.io/?id=geetanjali-salon</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123476?text=Hi%20Geetanjali%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Geetanjali%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dgeetanjali-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123476?text=Hi%20Geetanjali%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Geetanjali%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgeetanjali-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2212,12 +2212,12 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=looks-salon</t>
+          <t>https://reputetap.github.io/?id=looks-salon</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123477?text=Hi%20Looks%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Looks%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dlooks-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123477?text=Hi%20Looks%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Looks%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlooks-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=headmasters-salon</t>
+          <t>https://reputetap.github.io/?id=headmasters-salon</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123478?text=Hi%20Headmasters%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Headmasters%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dheadmasters-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123478?text=Hi%20Headmasters%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Headmasters%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dheadmasters-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2302,12 +2302,12 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=aura-thai-spa</t>
+          <t>https://reputetap.github.io/?id=aura-thai-spa</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123479?text=Hi%20Aura%20Thai%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Thai%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Daura-thai-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123479?text=Hi%20Aura%20Thai%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Thai%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-thai-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2347,12 +2347,12 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=o2-spa</t>
+          <t>https://reputetap.github.io/?id=o2-spa</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123480?text=Hi%20O2%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20O2%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Do2-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123480?text=Hi%20O2%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20O2%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Do2-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2392,12 +2392,12 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=tress-and-glow</t>
+          <t>https://reputetap.github.io/?id=tress-and-glow</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123481?text=Hi%20Tress%20%26%20Glow%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Tress%20%26%20Glow%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dtress-and-glow%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123481?text=Hi%20Tress%20%26%20Glow%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Tress%20%26%20Glow%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtress-and-glow%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=scissors-sound-salon</t>
+          <t>https://reputetap.github.io/?id=scissors-sound-salon</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123482?text=Hi%20Scissors%20Sound%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Scissors%20Sound%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dscissors-sound-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123482?text=Hi%20Scissors%20Sound%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Scissors%20Sound%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dscissors-sound-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=blush-and-bloom-makeovers</t>
+          <t>https://reputetap.github.io/?id=blush-and-bloom-makeovers</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123483?text=Hi%20Blush%20%26%20Bloom%20Makeovers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Blush%20%26%20Bloom%20Makeovers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dblush-and-bloom-makeovers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123483?text=Hi%20Blush%20%26%20Bloom%20Makeovers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Blush%20%26%20Bloom%20Makeovers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dblush-and-bloom-makeovers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=sizzling-scizzors</t>
+          <t>https://reputetap.github.io/?id=sizzling-scizzors</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123484?text=Hi%20Sizzling%20Scizzors%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sizzling%20Scizzors%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dsizzling-scizzors%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123484?text=Hi%20Sizzling%20Scizzors%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sizzling%20Scizzors%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsizzling-scizzors%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -2572,12 +2572,12 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=studio-99-salon-and-spa</t>
+          <t>https://reputetap.github.io/?id=studio-99-salon-and-spa</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123485?text=Hi%20Studio%2099%20Salon%20%26%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Studio%2099%20Salon%20%26%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dstudio-99-salon-and-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123485?text=Hi%20Studio%2099%20Salon%20%26%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Studio%2099%20Salon%20%26%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstudio-99-salon-and-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -2617,12 +2617,12 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-grooming-co</t>
+          <t>https://reputetap.github.io/?id=the-grooming-co</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123486?text=Hi%20The%20Grooming%20Co.%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Grooming%20Co.%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-grooming-co%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123486?text=Hi%20The%20Grooming%20Co.%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Grooming%20Co.%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-grooming-co%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -2662,12 +2662,12 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=envy-unisex-salon</t>
+          <t>https://reputetap.github.io/?id=envy-unisex-salon</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123487?text=Hi%20Envy%20Unisex%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Envy%20Unisex%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Denvy-unisex-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123487?text=Hi%20Envy%20Unisex%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Envy%20Unisex%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denvy-unisex-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -2707,12 +2707,12 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-detailing-mafia</t>
+          <t>https://reputetap.github.io/?id=the-detailing-mafia</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123488?text=Hi%20The%20Detailing%20Mafia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Detailing%20Mafia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-detailing-mafia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123488?text=Hi%20The%20Detailing%20Mafia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Detailing%20Mafia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-detailing-mafia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -2752,12 +2752,12 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=ceramic-pro-vadodara</t>
+          <t>https://reputetap.github.io/?id=ceramic-pro-vadodara</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123489?text=Hi%20Ceramic%20Pro%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ceramic%20Pro%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dceramic-pro-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123489?text=Hi%20Ceramic%20Pro%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ceramic%20Pro%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dceramic-pro-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=express-car-wash</t>
+          <t>https://reputetap.github.io/?id=express-car-wash</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123490?text=Hi%20Express%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Express%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dexpress-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123490?text=Hi%20Express%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Express%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dexpress-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=3m-car-care</t>
+          <t>https://reputetap.github.io/?id=3m-car-care</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123491?text=Hi%203M%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%203M%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3D3m-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123491?text=Hi%203M%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%203M%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D3m-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -2887,12 +2887,12 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=speed-car-wash</t>
+          <t>https://reputetap.github.io/?id=speed-car-wash</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123492?text=Hi%20Speed%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Speed%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dspeed-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123492?text=Hi%20Speed%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Speed%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dspeed-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=autoshine-detailing-studio</t>
+          <t>https://reputetap.github.io/?id=autoshine-detailing-studio</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123493?text=Hi%20Autoshine%20Detailing%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Autoshine%20Detailing%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dautoshine-detailing-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123493?text=Hi%20Autoshine%20Detailing%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Autoshine%20Detailing%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautoshine-detailing-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -2977,12 +2977,12 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=motoclean-studio</t>
+          <t>https://reputetap.github.io/?id=motoclean-studio</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123494?text=Hi%20MotoClean%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20MotoClean%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dmotoclean-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123494?text=Hi%20MotoClean%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20MotoClean%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmotoclean-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=torque-detailing-hub</t>
+          <t>https://reputetap.github.io/?id=torque-detailing-hub</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123495?text=Hi%20Torque%20Detailing%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Torque%20Detailing%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dtorque-detailing-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123495?text=Hi%20Torque%20Detailing%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Torque%20Detailing%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtorque-detailing-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
@@ -3067,12 +3067,12 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=gloss-autoworks</t>
+          <t>https://reputetap.github.io/?id=gloss-autoworks</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123496?text=Hi%20Gloss%20Autoworks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gloss%20Autoworks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dgloss-autoworks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123496?text=Hi%20Gloss%20Autoworks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gloss%20Autoworks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgloss-autoworks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -3112,12 +3112,12 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=carzspa-vadodara</t>
+          <t>https://reputetap.github.io/?id=carzspa-vadodara</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123497?text=Hi%20CarzSpa%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20CarzSpa%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcarzspa-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123497?text=Hi%20CarzSpa%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20CarzSpa%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcarzspa-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -3157,12 +3157,12 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=prime-auto-detailing</t>
+          <t>https://reputetap.github.io/?id=prime-auto-detailing</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123498?text=Hi%20Prime%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Prime%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dprime-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123498?text=Hi%20Prime%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Prime%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dprime-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
@@ -3202,12 +3202,12 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-car-lounge</t>
+          <t>https://reputetap.github.io/?id=the-car-lounge</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123499?text=Hi%20The%20Car%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Car%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-car-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123499?text=Hi%20The%20Car%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Car%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-car-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
@@ -3247,12 +3247,12 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=pitstop-car-spa</t>
+          <t>https://reputetap.github.io/?id=pitstop-car-spa</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123500?text=Hi%20Pitstop%20Car%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Pitstop%20Car%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dpitstop-car-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123500?text=Hi%20Pitstop%20Car%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Pitstop%20Car%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dpitstop-car-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
@@ -3292,12 +3292,12 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=royal-touch-car-care</t>
+          <t>https://reputetap.github.io/?id=royal-touch-car-care</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123501?text=Hi%20Royal%20Touch%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Royal%20Touch%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Droyal-touch-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123501?text=Hi%20Royal%20Touch%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Royal%20Touch%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Droyal-touch-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -3337,12 +3337,12 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=revive-auto-detailing</t>
+          <t>https://reputetap.github.io/?id=revive-auto-detailing</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123502?text=Hi%20Revive%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Revive%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Drevive-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123502?text=Hi%20Revive%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Revive%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Drevive-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -3382,12 +3382,12 @@
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=shieldpro-detailing</t>
+          <t>https://reputetap.github.io/?id=shieldpro-detailing</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123503?text=Hi%20ShieldPro%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ShieldPro%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dshieldpro-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123503?text=Hi%20ShieldPro%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ShieldPro%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshieldpro-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
@@ -3427,12 +3427,12 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=autogleam-car-wash</t>
+          <t>https://reputetap.github.io/?id=autogleam-car-wash</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123504?text=Hi%20AutoGleam%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoGleam%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dautogleam-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123504?text=Hi%20AutoGleam%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoGleam%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautogleam-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
@@ -3472,12 +3472,12 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=urban-auto-spa</t>
+          <t>https://reputetap.github.io/?id=urban-auto-spa</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123505?text=Hi%20Urban%20Auto%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Urban%20Auto%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Durban-auto-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123505?text=Hi%20Urban%20Auto%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Urban%20Auto%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Durban-auto-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
@@ -3517,12 +3517,12 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=apex-ceramic-lab</t>
+          <t>https://reputetap.github.io/?id=apex-ceramic-lab</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123506?text=Hi%20Apex%20Ceramic%20Lab%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Apex%20Ceramic%20Lab%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dapex-ceramic-lab%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123506?text=Hi%20Apex%20Ceramic%20Lab%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Apex%20Ceramic%20Lab%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dapex-ceramic-lab%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -3562,12 +3562,12 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=autowrap-studio</t>
+          <t>https://reputetap.github.io/?id=autowrap-studio</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123507?text=Hi%20AutoWrap%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoWrap%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dautowrap-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123507?text=Hi%20AutoWrap%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoWrap%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautowrap-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=smile-care-dental-clinic</t>
+          <t>https://reputetap.github.io/?id=smile-care-dental-clinic</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123508?text=Hi%20Smile%20Care%20Dental%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Smile%20Care%20Dental%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dsmile-care-dental-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123508?text=Hi%20Smile%20Care%20Dental%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Smile%20Care%20Dental%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsmile-care-dental-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -3652,12 +3652,12 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=32-pearls-dental-care</t>
+          <t>https://reputetap.github.io/?id=32-pearls-dental-care</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123509?text=Hi%2032%20Pearls%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2032%20Pearls%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3D32-pearls-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123509?text=Hi%2032%20Pearls%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2032%20Pearls%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D32-pearls-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
@@ -3697,12 +3697,12 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=baroda-dental-studio</t>
+          <t>https://reputetap.github.io/?id=baroda-dental-studio</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123510?text=Hi%20Baroda%20Dental%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Baroda%20Dental%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dbaroda-dental-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123510?text=Hi%20Baroda%20Dental%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Baroda%20Dental%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbaroda-dental-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -3742,12 +3742,12 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=dr-dhrutis-aesthetic-clinic</t>
+          <t>https://reputetap.github.io/?id=dr-dhrutis-aesthetic-clinic</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123511?text=Hi%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Ddr-dhrutis-aesthetic-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123511?text=Hi%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-dhrutis-aesthetic-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
@@ -3787,12 +3787,12 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=aura-skin-and-hair-clinic</t>
+          <t>https://reputetap.github.io/?id=aura-skin-and-hair-clinic</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123512?text=Hi%20Aura%20Skin%20%26%20Hair%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Skin%20%26%20Hair%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Daura-skin-and-hair-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123512?text=Hi%20Aura%20Skin%20%26%20Hair%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Skin%20%26%20Hair%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-skin-and-hair-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
@@ -3832,12 +3832,12 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-dental-hub</t>
+          <t>https://reputetap.github.io/?id=the-dental-hub</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123513?text=Hi%20The%20Dental%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dental%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-dental-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123513?text=Hi%20The%20Dental%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dental%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dental-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
@@ -3877,12 +3877,12 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=cosmodent-dental-care</t>
+          <t>https://reputetap.github.io/?id=cosmodent-dental-care</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123514?text=Hi%20Cosmodent%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cosmodent%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dcosmodent-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123514?text=Hi%20Cosmodent%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cosmodent%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcosmodent-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
@@ -3922,12 +3922,12 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=dermaelite-skin-studio</t>
+          <t>https://reputetap.github.io/?id=dermaelite-skin-studio</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123515?text=Hi%20DermaElite%20Skin%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20DermaElite%20Skin%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Ddermaelite-skin-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123515?text=Hi%20DermaElite%20Skin%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20DermaElite%20Skin%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddermaelite-skin-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
@@ -3967,12 +3967,12 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=dr-trivedi-dental-hospital</t>
+          <t>https://reputetap.github.io/?id=dr-trivedi-dental-hospital</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123516?text=Hi%20Dr.%20Trivedi%20Dental%20Hospital%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Trivedi%20Dental%20Hospital%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Ddr-trivedi-dental-hospital%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123516?text=Hi%20Dr.%20Trivedi%20Dental%20Hospital%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Trivedi%20Dental%20Hospital%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-trivedi-dental-hospital%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
@@ -4012,12 +4012,12 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=dentique-advanced-dental</t>
+          <t>https://reputetap.github.io/?id=dentique-advanced-dental</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123517?text=Hi%20Dentique%20Advanced%20Dental%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dentique%20Advanced%20Dental%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Ddentique-advanced-dental%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123517?text=Hi%20Dentique%20Advanced%20Dental%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dentique%20Advanced%20Dental%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddentique-advanced-dental%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
@@ -4057,12 +4057,12 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=clearsmile-orthodontics</t>
+          <t>https://reputetap.github.io/?id=clearsmile-orthodontics</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123518?text=Hi%20ClearSmile%20Orthodontics%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ClearSmile%20Orthodontics%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dclearsmile-orthodontics%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123518?text=Hi%20ClearSmile%20Orthodontics%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ClearSmile%20Orthodontics%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dclearsmile-orthodontics%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr">
@@ -4102,12 +4102,12 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=radiance-skin-clinic</t>
+          <t>https://reputetap.github.io/?id=radiance-skin-clinic</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123519?text=Hi%20Radiance%20Skin%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Radiance%20Skin%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dradiance-skin-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123519?text=Hi%20Radiance%20Skin%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Radiance%20Skin%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dradiance-skin-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
@@ -4147,12 +4147,12 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=perfect-smile-clinic</t>
+          <t>https://reputetap.github.io/?id=perfect-smile-clinic</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123520?text=Hi%20Perfect%20Smile%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Perfect%20Smile%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dperfect-smile-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123520?text=Hi%20Perfect%20Smile%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Perfect%20Smile%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dperfect-smile-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr">
@@ -4192,12 +4192,12 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=zenith-dental-care</t>
+          <t>https://reputetap.github.io/?id=zenith-dental-care</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123521?text=Hi%20Zenith%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zenith%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dzenith-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123521?text=Hi%20Zenith%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zenith%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzenith-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=dr-patels-aesthetic-smile</t>
+          <t>https://reputetap.github.io/?id=dr-patels-aesthetic-smile</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123522?text=Hi%20Dr.%20Patel%27s%20Aesthetic%20Smile%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Patel%27s%20Aesthetic%20Smile%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Ddr-patels-aesthetic-smile%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123522?text=Hi%20Dr.%20Patel%27s%20Aesthetic%20Smile%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Patel%27s%20Aesthetic%20Smile%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-patels-aesthetic-smile%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
@@ -4282,12 +4282,12 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=mrunalini-rao-studio</t>
+          <t>https://reputetap.github.io/?id=mrunalini-rao-studio</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123523?text=Hi%20Mrunalini%20Rao%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mrunalini%20Rao%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dmrunalini-rao-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123523?text=Hi%20Mrunalini%20Rao%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mrunalini%20Rao%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmrunalini-rao-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
@@ -4327,12 +4327,12 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=sutra-designer-boutique</t>
+          <t>https://reputetap.github.io/?id=sutra-designer-boutique</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123524?text=Hi%20Sutra%20Designer%20Boutique%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sutra%20Designer%20Boutique%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dsutra-designer-boutique%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123524?text=Hi%20Sutra%20Designer%20Boutique%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sutra%20Designer%20Boutique%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsutra-designer-boutique%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -4372,12 +4372,12 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=shyamal-and-bhumika-showcase</t>
+          <t>https://reputetap.github.io/?id=shyamal-and-bhumika-showcase</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123525?text=Hi%20Shyamal%20%26%20Bhumika%20Showcase%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Shyamal%20%26%20Bhumika%20Showcase%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dshyamal-and-bhumika-showcase%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123525?text=Hi%20Shyamal%20%26%20Bhumika%20Showcase%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Shyamal%20%26%20Bhumika%20Showcase%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshyamal-and-bhumika-showcase%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I89" s="4" t="inlineStr">
@@ -4417,12 +4417,12 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=kala-niketan-silks</t>
+          <t>https://reputetap.github.io/?id=kala-niketan-silks</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123526?text=Hi%20Kala%20Niketan%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kala%20Niketan%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dkala-niketan-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123526?text=Hi%20Kala%20Niketan%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kala%20Niketan%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkala-niketan-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr">
@@ -4462,12 +4462,12 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=the-raymond-shop-alkapuri</t>
+          <t>https://reputetap.github.io/?id=the-raymond-shop-alkapuri</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123527?text=Hi%20The%20Raymond%20Shop%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Raymond%20Shop%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dthe-raymond-shop-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123527?text=Hi%20The%20Raymond%20Shop%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Raymond%20Shop%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-raymond-shop-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I91" s="4" t="inlineStr">
@@ -4507,12 +4507,12 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=zaveri-brothers</t>
+          <t>https://reputetap.github.io/?id=zaveri-brothers</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123528?text=Hi%20Zaveri%20Brothers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zaveri%20Brothers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dzaveri-brothers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123528?text=Hi%20Zaveri%20Brothers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zaveri%20Brothers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzaveri-brothers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -4552,12 +4552,12 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=asopalav-vadodara</t>
+          <t>https://reputetap.github.io/?id=asopalav-vadodara</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123529?text=Hi%20Asopalav%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Asopalav%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dasopalav-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123529?text=Hi%20Asopalav%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Asopalav%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dasopalav-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
@@ -4597,12 +4597,12 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=manyavar-and-mohey</t>
+          <t>https://reputetap.github.io/?id=manyavar-and-mohey</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123530?text=Hi%20Manyavar%20%26%20Mohey%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Manyavar%20%26%20Mohey%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dmanyavar-and-mohey%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123530?text=Hi%20Manyavar%20%26%20Mohey%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Manyavar%20%26%20Mohey%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmanyavar-and-mohey%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
@@ -4642,12 +4642,12 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=fabindia-alkapuri</t>
+          <t>https://reputetap.github.io/?id=fabindia-alkapuri</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123531?text=Hi%20Fabindia%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fabindia%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dfabindia-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123531?text=Hi%20Fabindia%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fabindia%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfabindia-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -4687,12 +4687,12 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=jadeblue-bespoke-tailoring</t>
+          <t>https://reputetap.github.io/?id=jadeblue-bespoke-tailoring</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123532?text=Hi%20JadeBlue%20Bespoke%20Tailoring%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20JadeBlue%20Bespoke%20Tailoring%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Djadeblue-bespoke-tailoring%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123532?text=Hi%20JadeBlue%20Bespoke%20Tailoring%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20JadeBlue%20Bespoke%20Tailoring%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djadeblue-bespoke-tailoring%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=virasat-heritage-silks</t>
+          <t>https://reputetap.github.io/?id=virasat-heritage-silks</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123533?text=Hi%20Virasat%20Heritage%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Virasat%20Heritage%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dvirasat-heritage-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123533?text=Hi%20Virasat%20Heritage%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Virasat%20Heritage%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dvirasat-heritage-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
@@ -4777,12 +4777,12 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=label-anushree</t>
+          <t>https://reputetap.github.io/?id=label-anushree</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123534?text=Hi%20Label%20Anushree%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Label%20Anushree%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dlabel-anushree%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123534?text=Hi%20Label%20Anushree%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Label%20Anushree%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlabel-anushree%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I98" s="4" t="inlineStr">
@@ -4822,12 +4822,12 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=kalki-fashion-experience</t>
+          <t>https://reputetap.github.io/?id=kalki-fashion-experience</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123535?text=Hi%20Kalki%20Fashion%20Experience%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kalki%20Fashion%20Experience%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dkalki-fashion-experience%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123535?text=Hi%20Kalki%20Fashion%20Experience%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kalki%20Fashion%20Experience%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkalki-fashion-experience%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I99" s="4" t="inlineStr">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=raw-mango-studio</t>
+          <t>https://reputetap.github.io/?id=raw-mango-studio</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123536?text=Hi%20Raw%20Mango%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Raw%20Mango%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Draw-mango-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123536?text=Hi%20Raw%20Mango%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Raw%20Mango%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Draw-mango-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr">
@@ -4912,12 +4912,12 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>https://mehulnayaka1.github.io/reputetap/?id=ritu-kumar-flagship</t>
+          <t>https://reputetap.github.io/?id=ritu-kumar-flagship</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123537?text=Hi%20Ritu%20Kumar%20Flagship%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ritu%20Kumar%20Flagship%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Fmehulnayaka1.github.io%2Freputetap%2F%3Fid%3Dritu-kumar-flagship%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123537?text=Hi%20Ritu%20Kumar%20Flagship%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ritu%20Kumar%20Flagship%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dritu-kumar-flagship%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I101" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Update web app, leads sheet, WhatsApp templates, and sales script with ₹299 Vadodara Launch Promo (90% OFF for first 100 venues)
</commit_message>
<xml_diff>
--- a/ReputeTap - 100 Outreach Leads (Vadodara & Gujarat).xlsx
+++ b/ReputeTap - 100 Outreach Leads (Vadodara & Gujarat).xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/916359220791?text=Hi%20Curators%20Coffee%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Curators%20Coffee%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcurators-coffee%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/916359220791?text=Hi%20Curators%20Coffee%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Curators%20Coffee%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcurators-coffee%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825336364?text=Hi%20Kaffa%20Coffee%20Roasters%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kaffa%20Coffee%20Roasters%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkaffa-coffee-roasters%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825336364?text=Hi%20Kaffa%20Coffee%20Roasters%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kaffa%20Coffee%20Roasters%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkaffa-coffee-roasters%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919978623256?text=Hi%20The%20Coffee%20Next%20Door%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Coffee%20Next%20Door%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-coffee-next-door%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919978623256?text=Hi%20The%20Coffee%20Next%20Door%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Coffee%20Next%20Door%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-coffee-next-door%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919773050954?text=Hi%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcharmant-the-heritage-caf%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919773050954?text=Hi%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Charmant%20%E2%80%93%20The%20Heritage%20Caf%C3%A9%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcharmant-the-heritage-caf%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/916357575811?text=Hi%20Burgundy%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Burgundy%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dburgundy-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/916357575811?text=Hi%20Burgundy%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Burgundy%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dburgundy-cafe%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919712348900?text=Hi%20Trinity%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Trinity%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtrinity-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919712348900?text=Hi%20Trinity%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Trinity%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtrinity-cafe%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123451?text=Hi%20The%20Dark%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dark%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dark-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123451?text=Hi%20The%20Dark%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dark%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dark-roast%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123452?text=Hi%20Brew%20Artisan%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Brew%20Artisan%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbrew-artisan-cafe%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123452?text=Hi%20Brew%20Artisan%20Cafe%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Brew%20Artisan%20Cafe%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbrew-artisan-cafe%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123453?text=Hi%20Mocha%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mocha%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmocha-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123453?text=Hi%20Mocha%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mocha%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmocha-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123454?text=Hi%20Cafe%20Fitoor%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cafe%20Fitoor%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcafe-fitoor%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123454?text=Hi%20Cafe%20Fitoor%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cafe%20Fitoor%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcafe-fitoor%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123455?text=Hi%20The%20Secret%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Secret%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-secret-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123455?text=Hi%20The%20Secret%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Secret%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-secret-kitchen%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123456?text=Hi%20Kai%20Asia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kai%20Asia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkai-asia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123456?text=Hi%20Kai%20Asia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kai%20Asia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkai-asia%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123457?text=Hi%20Gazebo%20Garden%20Restaurant%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gazebo%20Garden%20Restaurant%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgazebo-garden-restaurant%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123457?text=Hi%20Gazebo%20Garden%20Restaurant%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gazebo%20Garden%20Restaurant%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgazebo-garden-restaurant%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123458?text=Hi%20Little%20Italy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Little%20Italy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlittle-italy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123458?text=Hi%20Little%20Italy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Little%20Italy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlittle-italy%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123459?text=Hi%2022nd%20Parallel%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2022nd%20Parallel%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D22nd-parallel%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123459?text=Hi%2022nd%20Parallel%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2022nd%20Parallel%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D22nd-parallel%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123460?text=Hi%20Salsa%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Salsa%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsalsa-kitchen%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123460?text=Hi%20Salsa%20Kitchen%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Salsa%20Kitchen%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsalsa-kitchen%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123461?text=Hi%20Barbeque%20Nation%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Barbeque%20Nation%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbarbeque-nation%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123461?text=Hi%20Barbeque%20Nation%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Barbeque%20Nation%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbarbeque-nation%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123462?text=Hi%20That%20Place%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20That%20Place%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthat-place%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123462?text=Hi%20That%20Place%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20That%20Place%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthat-place%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123463?text=Hi%20Fresh%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fresh%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfresh-roast%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123463?text=Hi%20Fresh%20Roast%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fresh%20Roast%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfresh-roast%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123464?text=Hi%20Coffee%20Culture%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Coffee%20Culture%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcoffee-culture%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123464?text=Hi%20Coffee%20Culture%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Coffee%20Culture%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcoffee-culture%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123465?text=Hi%20Chai%20Sutta%20Bar%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Chai%20Sutta%20Bar%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchai-sutta-bar%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123465?text=Hi%20Chai%20Sutta%20Bar%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Chai%20Sutta%20Bar%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchai-sutta-bar%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123466?text=Hi%20Keventers%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Keventers%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkeventers-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123466?text=Hi%20Keventers%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Keventers%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkeventers-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123467?text=Hi%20Crust%20%26%20Crumbs%20Patisserie%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Crust%20%26%20Crumbs%20Patisserie%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcrust-and-crumbs-patisserie%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123467?text=Hi%20Crust%20%26%20Crumbs%20Patisserie%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Crust%20%26%20Crumbs%20Patisserie%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcrust-and-crumbs-patisserie%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123468?text=Hi%20Bake%20My%20Day%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bake%20My%20Day%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbake-my-day%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123468?text=Hi%20Bake%20My%20Day%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bake%20My%20Day%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbake-my-day%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123469?text=Hi%20The%20Chocolate%20Room%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Chocolate%20Room%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-chocolate-room%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123469?text=Hi%20The%20Chocolate%20Room%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Chocolate%20Room%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-chocolate-room%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919974098750?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio-and-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919974098750?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20%26%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio-and-lounge%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917600088148?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/917600088148?text=Hi%20Styloria%20Unisex%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Styloria%20Unisex%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstyloria-unisex-hair-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919152253000?text=Hi%20Enrich%20Salon%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Enrich%20Salon%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denrich-salon-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919152253000?text=Hi%20Enrich%20Salon%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Enrich%20Salon%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denrich-salon-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918238307599?text=Hi%20Wave%20Salon%20%26%20Academy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Wave%20Salon%20%26%20Academy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dwave-salon-and-academy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/918238307599?text=Hi%20Wave%20Salon%20%26%20Academy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Wave%20Salon%20%26%20Academy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dwave-salon-and-academy%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918291128445?text=Hi%20Lakme%20Salon%20For%20Him%20%26%20Her%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Lakme%20Salon%20For%20Him%20%26%20Her%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlakme-salon-for-him-and-her%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/918291128445?text=Hi%20Lakme%20Salon%20For%20Him%20%26%20Her%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Lakme%20Salon%20For%20Him%20%26%20Her%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlakme-salon-for-him-and-her%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/912652323222?text=Hi%20Cutz%20Beauty%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cutz%20Beauty%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcutz-beauty-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/912652323222?text=Hi%20Cutz%20Beauty%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cutz%20Beauty%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcutz-beauty-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919724661172?text=Hi%20Champion%20Ladies%20%26%20Gents%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Champion%20Ladies%20%26%20Gents%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchampion-ladies-and-gents-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919724661172?text=Hi%20Champion%20Ladies%20%26%20Gents%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Champion%20Ladies%20%26%20Gents%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dchampion-ladies-and-gents-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123470?text=Hi%20Truefitt%20%26%20Hill%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Truefitt%20%26%20Hill%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtruefitt-and-hill%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123470?text=Hi%20Truefitt%20%26%20Hill%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Truefitt%20%26%20Hill%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtruefitt-and-hill%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123471?text=Hi%20Toni%20%26%20Guy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Toni%20%26%20Guy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtoni-and-guy%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123471?text=Hi%20Toni%20%26%20Guy%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Toni%20%26%20Guy%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtoni-and-guy%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123472?text=Hi%20Jawed%20Habib%20Hair%20%26%20Beauty%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Jawed%20Habib%20Hair%20%26%20Beauty%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djawed-habib-hair-and-beauty%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123472?text=Hi%20Jawed%20Habib%20Hair%20%26%20Beauty%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Jawed%20Habib%20Hair%20%26%20Beauty%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djawed-habib-hair-and-beauty%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123473?text=Hi%20Bespoke%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bespoke%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbespoke-hair-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123473?text=Hi%20Bespoke%20Hair%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Bespoke%20Hair%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbespoke-hair-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123474?text=Hi%20The%20Nail%20Room%20Baroda%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Nail%20Room%20Baroda%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-nail-room-baroda%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123474?text=Hi%20The%20Nail%20Room%20Baroda%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Nail%20Room%20Baroda%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-nail-room-baroda%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123475?text=Hi%20Glam%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Glam%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dglam-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123475?text=Hi%20Glam%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Glam%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dglam-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123476?text=Hi%20Geetanjali%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Geetanjali%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgeetanjali-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123476?text=Hi%20Geetanjali%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Geetanjali%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgeetanjali-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123477?text=Hi%20Looks%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Looks%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlooks-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123477?text=Hi%20Looks%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Looks%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlooks-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123478?text=Hi%20Headmasters%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Headmasters%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dheadmasters-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123478?text=Hi%20Headmasters%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Headmasters%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dheadmasters-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123479?text=Hi%20Aura%20Thai%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Thai%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-thai-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123479?text=Hi%20Aura%20Thai%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Thai%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-thai-spa%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123480?text=Hi%20O2%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20O2%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Do2-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123480?text=Hi%20O2%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20O2%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Do2-spa%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123481?text=Hi%20Tress%20%26%20Glow%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Tress%20%26%20Glow%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtress-and-glow%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123481?text=Hi%20Tress%20%26%20Glow%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Tress%20%26%20Glow%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtress-and-glow%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123482?text=Hi%20Scissors%20Sound%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Scissors%20Sound%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dscissors-sound-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123482?text=Hi%20Scissors%20Sound%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Scissors%20Sound%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dscissors-sound-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123483?text=Hi%20Blush%20%26%20Bloom%20Makeovers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Blush%20%26%20Bloom%20Makeovers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dblush-and-bloom-makeovers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123483?text=Hi%20Blush%20%26%20Bloom%20Makeovers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Blush%20%26%20Bloom%20Makeovers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dblush-and-bloom-makeovers%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123484?text=Hi%20Sizzling%20Scizzors%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sizzling%20Scizzors%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsizzling-scizzors%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123484?text=Hi%20Sizzling%20Scizzors%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sizzling%20Scizzors%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsizzling-scizzors%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123485?text=Hi%20Studio%2099%20Salon%20%26%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Studio%2099%20Salon%20%26%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstudio-99-salon-and-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123485?text=Hi%20Studio%2099%20Salon%20%26%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Studio%2099%20Salon%20%26%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dstudio-99-salon-and-spa%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123486?text=Hi%20The%20Grooming%20Co.%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Grooming%20Co.%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-grooming-co%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123486?text=Hi%20The%20Grooming%20Co.%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Grooming%20Co.%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-grooming-co%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123487?text=Hi%20Envy%20Unisex%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Envy%20Unisex%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denvy-unisex-salon%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123487?text=Hi%20Envy%20Unisex%20Salon%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Envy%20Unisex%20Salon%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Denvy-unisex-salon%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123488?text=Hi%20The%20Detailing%20Mafia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Detailing%20Mafia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-detailing-mafia%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123488?text=Hi%20The%20Detailing%20Mafia%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Detailing%20Mafia%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-detailing-mafia%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123489?text=Hi%20Ceramic%20Pro%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ceramic%20Pro%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dceramic-pro-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123489?text=Hi%20Ceramic%20Pro%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ceramic%20Pro%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dceramic-pro-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123490?text=Hi%20Express%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Express%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dexpress-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123490?text=Hi%20Express%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Express%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dexpress-car-wash%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123491?text=Hi%203M%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%203M%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D3m-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123491?text=Hi%203M%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%203M%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D3m-car-care%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123492?text=Hi%20Speed%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Speed%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dspeed-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123492?text=Hi%20Speed%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Speed%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dspeed-car-wash%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123493?text=Hi%20Autoshine%20Detailing%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Autoshine%20Detailing%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautoshine-detailing-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123493?text=Hi%20Autoshine%20Detailing%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Autoshine%20Detailing%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautoshine-detailing-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123494?text=Hi%20MotoClean%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20MotoClean%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmotoclean-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123494?text=Hi%20MotoClean%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20MotoClean%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmotoclean-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123495?text=Hi%20Torque%20Detailing%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Torque%20Detailing%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtorque-detailing-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123495?text=Hi%20Torque%20Detailing%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Torque%20Detailing%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dtorque-detailing-hub%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123496?text=Hi%20Gloss%20Autoworks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gloss%20Autoworks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgloss-autoworks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123496?text=Hi%20Gloss%20Autoworks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Gloss%20Autoworks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dgloss-autoworks%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123497?text=Hi%20CarzSpa%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20CarzSpa%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcarzspa-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123497?text=Hi%20CarzSpa%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20CarzSpa%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcarzspa-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123498?text=Hi%20Prime%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Prime%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dprime-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123498?text=Hi%20Prime%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Prime%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dprime-auto-detailing%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123499?text=Hi%20The%20Car%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Car%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-car-lounge%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123499?text=Hi%20The%20Car%20Lounge%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Car%20Lounge%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-car-lounge%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123500?text=Hi%20Pitstop%20Car%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Pitstop%20Car%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dpitstop-car-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123500?text=Hi%20Pitstop%20Car%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Pitstop%20Car%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dpitstop-car-spa%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123501?text=Hi%20Royal%20Touch%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Royal%20Touch%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Droyal-touch-car-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123501?text=Hi%20Royal%20Touch%20Car%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Royal%20Touch%20Car%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Droyal-touch-car-care%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123502?text=Hi%20Revive%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Revive%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Drevive-auto-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123502?text=Hi%20Revive%20Auto%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Revive%20Auto%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Drevive-auto-detailing%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123503?text=Hi%20ShieldPro%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ShieldPro%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshieldpro-detailing%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123503?text=Hi%20ShieldPro%20Detailing%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ShieldPro%20Detailing%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshieldpro-detailing%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123504?text=Hi%20AutoGleam%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoGleam%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautogleam-car-wash%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123504?text=Hi%20AutoGleam%20Car%20Wash%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoGleam%20Car%20Wash%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautogleam-car-wash%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123505?text=Hi%20Urban%20Auto%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Urban%20Auto%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Durban-auto-spa%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123505?text=Hi%20Urban%20Auto%20Spa%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Urban%20Auto%20Spa%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Durban-auto-spa%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123506?text=Hi%20Apex%20Ceramic%20Lab%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Apex%20Ceramic%20Lab%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dapex-ceramic-lab%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123506?text=Hi%20Apex%20Ceramic%20Lab%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Apex%20Ceramic%20Lab%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dapex-ceramic-lab%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123507?text=Hi%20AutoWrap%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoWrap%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautowrap-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123507?text=Hi%20AutoWrap%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20AutoWrap%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dautowrap-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123508?text=Hi%20Smile%20Care%20Dental%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Smile%20Care%20Dental%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsmile-care-dental-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123508?text=Hi%20Smile%20Care%20Dental%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Smile%20Care%20Dental%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsmile-care-dental-clinic%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123509?text=Hi%2032%20Pearls%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2032%20Pearls%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D32-pearls-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123509?text=Hi%2032%20Pearls%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%2032%20Pearls%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3D32-pearls-dental-care%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123510?text=Hi%20Baroda%20Dental%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Baroda%20Dental%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbaroda-dental-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123510?text=Hi%20Baroda%20Dental%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Baroda%20Dental%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dbaroda-dental-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123511?text=Hi%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-dhrutis-aesthetic-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123511?text=Hi%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Dhruti%27s%20Aesthetic%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-dhrutis-aesthetic-clinic%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123512?text=Hi%20Aura%20Skin%20%26%20Hair%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Skin%20%26%20Hair%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-skin-and-hair-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123512?text=Hi%20Aura%20Skin%20%26%20Hair%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Aura%20Skin%20%26%20Hair%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Daura-skin-and-hair-clinic%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123513?text=Hi%20The%20Dental%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dental%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dental-hub%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123513?text=Hi%20The%20Dental%20Hub%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Dental%20Hub%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-dental-hub%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123514?text=Hi%20Cosmodent%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cosmodent%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcosmodent-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123514?text=Hi%20Cosmodent%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Cosmodent%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dcosmodent-dental-care%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123515?text=Hi%20DermaElite%20Skin%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20DermaElite%20Skin%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddermaelite-skin-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123515?text=Hi%20DermaElite%20Skin%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20DermaElite%20Skin%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddermaelite-skin-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123516?text=Hi%20Dr.%20Trivedi%20Dental%20Hospital%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Trivedi%20Dental%20Hospital%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-trivedi-dental-hospital%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123516?text=Hi%20Dr.%20Trivedi%20Dental%20Hospital%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Trivedi%20Dental%20Hospital%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-trivedi-dental-hospital%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123517?text=Hi%20Dentique%20Advanced%20Dental%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dentique%20Advanced%20Dental%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddentique-advanced-dental%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123517?text=Hi%20Dentique%20Advanced%20Dental%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dentique%20Advanced%20Dental%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddentique-advanced-dental%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123518?text=Hi%20ClearSmile%20Orthodontics%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ClearSmile%20Orthodontics%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dclearsmile-orthodontics%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123518?text=Hi%20ClearSmile%20Orthodontics%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20ClearSmile%20Orthodontics%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dclearsmile-orthodontics%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123519?text=Hi%20Radiance%20Skin%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Radiance%20Skin%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dradiance-skin-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123519?text=Hi%20Radiance%20Skin%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Radiance%20Skin%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dradiance-skin-clinic%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123520?text=Hi%20Perfect%20Smile%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Perfect%20Smile%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dperfect-smile-clinic%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123520?text=Hi%20Perfect%20Smile%20Clinic%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Perfect%20Smile%20Clinic%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dperfect-smile-clinic%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123521?text=Hi%20Zenith%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zenith%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzenith-dental-care%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123521?text=Hi%20Zenith%20Dental%20Care%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zenith%20Dental%20Care%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzenith-dental-care%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123522?text=Hi%20Dr.%20Patel%27s%20Aesthetic%20Smile%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Patel%27s%20Aesthetic%20Smile%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-patels-aesthetic-smile%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123522?text=Hi%20Dr.%20Patel%27s%20Aesthetic%20Smile%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Dr.%20Patel%27s%20Aesthetic%20Smile%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Ddr-patels-aesthetic-smile%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123523?text=Hi%20Mrunalini%20Rao%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mrunalini%20Rao%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmrunalini-rao-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123523?text=Hi%20Mrunalini%20Rao%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Mrunalini%20Rao%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmrunalini-rao-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123524?text=Hi%20Sutra%20Designer%20Boutique%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sutra%20Designer%20Boutique%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsutra-designer-boutique%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123524?text=Hi%20Sutra%20Designer%20Boutique%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Sutra%20Designer%20Boutique%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dsutra-designer-boutique%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123525?text=Hi%20Shyamal%20%26%20Bhumika%20Showcase%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Shyamal%20%26%20Bhumika%20Showcase%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshyamal-and-bhumika-showcase%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123525?text=Hi%20Shyamal%20%26%20Bhumika%20Showcase%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Shyamal%20%26%20Bhumika%20Showcase%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dshyamal-and-bhumika-showcase%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I89" s="4" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123526?text=Hi%20Kala%20Niketan%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kala%20Niketan%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkala-niketan-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123526?text=Hi%20Kala%20Niketan%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kala%20Niketan%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkala-niketan-silks%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123527?text=Hi%20The%20Raymond%20Shop%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Raymond%20Shop%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-raymond-shop-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123527?text=Hi%20The%20Raymond%20Shop%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20The%20Raymond%20Shop%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dthe-raymond-shop-alkapuri%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I91" s="4" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123528?text=Hi%20Zaveri%20Brothers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zaveri%20Brothers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzaveri-brothers%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123528?text=Hi%20Zaveri%20Brothers%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Zaveri%20Brothers%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dzaveri-brothers%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123529?text=Hi%20Asopalav%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Asopalav%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dasopalav-vadodara%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123529?text=Hi%20Asopalav%20Vadodara%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Asopalav%20Vadodara%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dasopalav-vadodara%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123530?text=Hi%20Manyavar%20%26%20Mohey%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Manyavar%20%26%20Mohey%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmanyavar-and-mohey%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123530?text=Hi%20Manyavar%20%26%20Mohey%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Manyavar%20%26%20Mohey%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dmanyavar-and-mohey%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123531?text=Hi%20Fabindia%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fabindia%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfabindia-alkapuri%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123531?text=Hi%20Fabindia%20Alkapuri%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Fabindia%20Alkapuri%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dfabindia-alkapuri%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123532?text=Hi%20JadeBlue%20Bespoke%20Tailoring%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20JadeBlue%20Bespoke%20Tailoring%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djadeblue-bespoke-tailoring%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123532?text=Hi%20JadeBlue%20Bespoke%20Tailoring%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20JadeBlue%20Bespoke%20Tailoring%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Djadeblue-bespoke-tailoring%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123533?text=Hi%20Virasat%20Heritage%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Virasat%20Heritage%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dvirasat-heritage-silks%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123533?text=Hi%20Virasat%20Heritage%20Silks%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Virasat%20Heritage%20Silks%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dvirasat-heritage-silks%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123534?text=Hi%20Label%20Anushree%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Label%20Anushree%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlabel-anushree%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123534?text=Hi%20Label%20Anushree%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Label%20Anushree%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dlabel-anushree%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I98" s="4" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123535?text=Hi%20Kalki%20Fashion%20Experience%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kalki%20Fashion%20Experience%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkalki-fashion-experience%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123535?text=Hi%20Kalki%20Fashion%20Experience%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Kalki%20Fashion%20Experience%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dkalki-fashion-experience%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I99" s="4" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123536?text=Hi%20Raw%20Mango%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Raw%20Mango%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Draw-mango-studio%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123536?text=Hi%20Raw%20Mango%20Studio%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Raw%20Mango%20Studio%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Draw-mango-studio%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/919825123537?text=Hi%20Ritu%20Kumar%20Flagship%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ritu%20Kumar%20Flagship%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dritu-kumar-flagship%0A%0AWe%20deliver%202%20custom%20standees%20with%20your%20logo%20and%20zero%20monthly%20software%20fees.%20Would%20you%20like%20us%20to%20drop%20off%20a%20sample%20at%20your%20counter%20this%20week%3F</t>
+          <t>https://wa.me/919825123537?text=Hi%20Ritu%20Kumar%20Flagship%20Team%21%20%F0%9F%91%8B%20Quick%2010-second%20message%20from%20Vadodara%3A%0A%0AWe%20are%20manufacturing%20custom%20laser-cut%20acrylic%20NFC%20counter%20standees%20for%20local%20businesses%20in%20Vadodara%20to%20solve%20checkout%20review%20friction.%0A%0ARight%20now%2C%2090%25%2B%20of%20happy%20visitors%20at%20Ritu%20Kumar%20Flagship%20walk%20out%20without%20reviewing%20on%20Google%20because%20searching%20and%20typing%20takes%20too%20long.%20With%20this%20standee%20on%20your%20billing%20counter%3A%0A1.%20Customers%20tap%20their%20phone%20%28or%20scan%20QR%29%20and%20our%201-tap%20assistant%20drafts%20a%205-star%20review%20in%202%20seconds.%0A2.%20If%20someone%20had%20an%20issue%2C%20it%20routes%20feedback%20privately%20to%20your%20WhatsApp%20so%20you%20can%20fix%20it%20on%20the%20spot%20before%20a%201-star%20review%20goes%20public.%0A%0AI%20pre-programmed%20a%2010-second%20interactive%20digital%20simulation%20of%20your%20custom%20standee%20here%20so%20you%20can%20test%20it%20on%20your%20phone%3A%0A%F0%9F%91%89%20https%3A%2F%2Freputetap.github.io%2F%3Fid%3Dritu-kumar-flagship%0A%0A%F0%9F%94%A5%20VADODARA%20LAUNCH%20PROMO%3A%20We%20are%20delivering%202%20custom-branded%20standees%20with%20your%20logo%20for%20just%20%E2%82%B9299%20%28Regular%20%E2%82%B92%2C999%29%20for%20our%20first%20100%20partner%20venues%21%0A%0AWould%20you%20like%20us%20to%20drop%20off%20a%20sample%20set%20at%20your%20counter%20this%20week%3F</t>
         </is>
       </c>
       <c r="I101" s="4" t="inlineStr">

</xml_diff>